<commit_message>
Randomize 2027 test data)
</commit_message>
<xml_diff>
--- a/data/Carlson Creek Restoration/Lower Stream/Site 3/IS 3/Site3, #10, 22449418 2027-02-27 16_38_33 PST (Data PST).xlsx
+++ b/data/Carlson Creek Restoration/Lower Stream/Site 3/IS 3/Site3, #10, 22449418 2027-02-27 16_38_33 PST (Data PST).xlsx
@@ -511,10 +511,10 @@
         <v>46444.45833333334</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>4.470279693603516</v>
+        <v>5.162</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>94.12286343448243</v>
+        <v>95.184</v>
       </c>
     </row>
     <row r="3">
@@ -525,10 +525,10 @@
         <v>46444.5</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5.573917388916016</v>
+        <v>5.959</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>94.0514156493785</v>
+        <v>95.178</v>
       </c>
     </row>
     <row r="4">
@@ -539,10 +539,10 @@
         <v>46444.54166666666</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3.071414709091187</v>
+        <v>3.524</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>96.35563630806854</v>
+        <v>97.611</v>
       </c>
     </row>
     <row r="5">
@@ -553,10 +553,10 @@
         <v>46444.58333333334</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3.084659337997437</v>
+        <v>3.477</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>96.31900501681011</v>
+        <v>97.45399999999999</v>
       </c>
     </row>
     <row r="6">
@@ -567,10 +567,10 @@
         <v>46444.625</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3.233493566513062</v>
+        <v>3.839</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>96.31279788362973</v>
+        <v>97.517</v>
       </c>
     </row>
     <row r="7">
@@ -581,10 +581,10 @@
         <v>46444.66666666666</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3.382022619247437</v>
+        <v>3.798</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>96.24588709205807</v>
+        <v>97.34699999999999</v>
       </c>
     </row>
     <row r="8">
@@ -595,10 +595,10 @@
         <v>46444.70833333334</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3.349063634872437</v>
+        <v>4.249</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>96.23951557505404</v>
+        <v>97.40900000000001</v>
       </c>
     </row>
     <row r="9">
@@ -609,10 +609,10 @@
         <v>46444.75</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.312747716903687</v>
+        <v>3.608</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>96.28893592779113</v>
+        <v>97.34</v>
       </c>
     </row>
     <row r="10">
@@ -623,10 +623,10 @@
         <v>46444.79166666666</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.220279455184937</v>
+        <v>3.672</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>96.30743897097929</v>
+        <v>97.462</v>
       </c>
     </row>
     <row r="11">
@@ -637,10 +637,10 @@
         <v>46444.83333333334</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>3.188876867294312</v>
+        <v>4.027</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>96.34777876129887</v>
+        <v>97.59399999999999</v>
       </c>
     </row>
     <row r="12">
@@ -651,10 +651,10 @@
         <v>46444.875</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3.134311437606812</v>
+        <v>3.556</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>96.39158376262064</v>
+        <v>97.76600000000001</v>
       </c>
     </row>
     <row r="13">
@@ -665,10 +665,10 @@
         <v>46444.91666666666</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3.091281652450562</v>
+        <v>3.76</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>96.40798926821924</v>
+        <v>97.57899999999999</v>
       </c>
     </row>
     <row r="14">
@@ -679,10 +679,10 @@
         <v>46444.95833333334</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>3.031680822372437</v>
+        <v>3.548</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>96.38621169926431</v>
+        <v>97.605</v>
       </c>
     </row>
     <row r="15">
@@ -693,10 +693,10 @@
         <v>46445</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>2.968662023544312</v>
+        <v>3.362</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>96.37824237149458</v>
+        <v>97.432</v>
       </c>
     </row>
     <row r="16">
@@ -707,10 +707,10 @@
         <v>46445.04166666666</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>2.928867101669312</v>
+        <v>3.585</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>96.40880461198445</v>
+        <v>97.48099999999999</v>
       </c>
     </row>
     <row r="17">
@@ -721,10 +721,10 @@
         <v>46445.08333333334</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>2.892368078231812</v>
+        <v>3.128</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>96.397554183095</v>
+        <v>97.639</v>
       </c>
     </row>
     <row r="18">
@@ -735,10 +735,10 @@
         <v>46445.125</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>2.829257726669312</v>
+        <v>3.603</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>96.3522500013017</v>
+        <v>97.55800000000001</v>
       </c>
     </row>
     <row r="19">
@@ -749,10 +749,10 @@
         <v>46445.16666666666</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2.781039953231812</v>
+        <v>3.215</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>96.3450565651795</v>
+        <v>97.446</v>
       </c>
     </row>
     <row r="20">
@@ -763,10 +763,10 @@
         <v>46445.20833333334</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2.746127843856812</v>
+        <v>3.368</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>96.34787739159304</v>
+        <v>97.517</v>
       </c>
     </row>
     <row r="21">
@@ -777,10 +777,10 @@
         <v>46445.25</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.692874670028687</v>
+        <v>3.28</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>96.38237826849718</v>
+        <v>97.506</v>
       </c>
     </row>
     <row r="22">
@@ -791,10 +791,10 @@
         <v>46445.29166666666</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2.646213293075562</v>
+        <v>3.155</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>96.39856678744859</v>
+        <v>97.384</v>
       </c>
     </row>
     <row r="23">
@@ -805,10 +805,10 @@
         <v>46445.33333333334</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2.614566564559937</v>
+        <v>3.132</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>96.39224787326812</v>
+        <v>97.642</v>
       </c>
     </row>
     <row r="24">
@@ -819,10 +819,10 @@
         <v>46445.375</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>2.609561681747437</v>
+        <v>3.351</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>96.382641282615</v>
+        <v>97.515</v>
       </c>
     </row>
     <row r="25">
@@ -833,10 +833,10 @@
         <v>46445.41666666666</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>2.642886877059937</v>
+        <v>3.088</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>96.32377872304842</v>
+        <v>97.276</v>
       </c>
     </row>
     <row r="26">
@@ -847,10 +847,10 @@
         <v>46445.45833333334</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>2.701205968856812</v>
+        <v>3.064</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>96.34084176394155</v>
+        <v>97.48099999999999</v>
       </c>
     </row>
     <row r="27">
@@ -861,10 +861,10 @@
         <v>46445.5</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2.792667150497437</v>
+        <v>3.427</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>96.34100614776519</v>
+        <v>97.511</v>
       </c>
     </row>
     <row r="28">
@@ -875,10 +875,10 @@
         <v>46445.54166666666</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2.895663976669312</v>
+        <v>3.457</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>96.30910253527445</v>
+        <v>97.602</v>
       </c>
     </row>
     <row r="29">
@@ -889,10 +889,10 @@
         <v>46445.58333333334</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>3.049869298934937</v>
+        <v>3.64</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>96.31252171880602</v>
+        <v>97.36199999999999</v>
       </c>
     </row>
     <row r="30">
@@ -903,10 +903,10 @@
         <v>46445.625</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>3.109500646591187</v>
+        <v>3.784</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>96.29232223455797</v>
+        <v>97.33199999999999</v>
       </c>
     </row>
     <row r="31">
@@ -917,10 +917,10 @@
         <v>46445.66666666666</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>3.160770177841187</v>
+        <v>3.565</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>96.25302135000375</v>
+        <v>97.383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>